<commit_message>
comments updated, implemented Doxygen
</commit_message>
<xml_diff>
--- a/Documents/UDP Packet Structure.xlsx
+++ b/Documents/UDP Packet Structure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\University Work\3rd Year\3rd Year Project\University-3rd-Year-Project\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26AFA82C-7741-4806-B462-45222CC9E5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A68E35C-FD0C-44EC-AC65-1D516E4251E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{1ADFE77D-9655-4730-AA72-896D6228A30D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{1ADFE77D-9655-4730-AA72-896D6228A30D}"/>
   </bookViews>
   <sheets>
     <sheet name="Packet Information" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="62">
   <si>
     <t>Name</t>
   </si>
@@ -126,9 +126,6 @@
     <t>Header Version</t>
   </si>
   <si>
-    <t>Message counter (incremented by ack requester)</t>
-  </si>
-  <si>
     <t>Data is little endian</t>
   </si>
   <si>
@@ -219,7 +216,13 @@
     <t>02 B5 00 0E 00 00 00 00 01 23 45 67 89 AB CD EF 00 00 00 00 00 00 00 01 00 00 01 97 2B C5 80 00 00 00 00 64 01 01 00 01 01 00 0A 00 52 CF 22 41 01 02 03 04 05 06 07 08 11 22 33 44 55 66 5B 03</t>
   </si>
   <si>
-    <t>ESP Type</t>
+    <t>Packet Type</t>
+  </si>
+  <si>
+    <t>Destination UID</t>
+  </si>
+  <si>
+    <t>Forwarding Mode</t>
   </si>
 </sst>
 </file>
@@ -821,7 +824,7 @@
     </row>
     <row r="2" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C2" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D2" s="13"/>
       <c r="E2" s="14"/>
@@ -887,7 +890,7 @@
         <v>2</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="10">
@@ -916,7 +919,7 @@
         <v>2</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F6" s="4"/>
       <c r="G6" s="10">
@@ -959,7 +962,7 @@
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
@@ -974,7 +977,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F8" s="4"/>
       <c r="G8" s="10">
@@ -988,7 +991,7 @@
       </c>
       <c r="J8" s="4"/>
       <c r="K8" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
@@ -1003,7 +1006,7 @@
         <v>8</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="F9" s="4"/>
       <c r="G9" s="10">
@@ -1044,7 +1047,7 @@
       </c>
       <c r="J10" s="4"/>
       <c r="K10" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
@@ -1073,7 +1076,7 @@
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
@@ -1113,7 +1116,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
@@ -1154,14 +1157,14 @@
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H15" s="4"/>
       <c r="I15" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="3:14" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -1173,18 +1176,18 @@
         <v>1</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F16" s="4"/>
       <c r="G16" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H16" s="4"/>
       <c r="I16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="J16" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="17" spans="3:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -1196,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F17" s="4"/>
       <c r="H17" s="4"/>
@@ -1211,7 +1214,7 @@
         <v>1</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F18" s="4"/>
       <c r="H18" s="4"/>
@@ -1226,7 +1229,7 @@
         <v>1</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="F19" s="4"/>
       <c r="H19" s="4"/>
@@ -1332,7 +1335,7 @@
     </row>
     <row r="29" spans="3:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C29" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D29" s="13"/>
       <c r="E29" s="14"/>
@@ -1373,7 +1376,7 @@
         <v>2</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F32" s="4"/>
       <c r="G32" s="4"/>
@@ -1442,7 +1445,7 @@
     </row>
     <row r="39" spans="3:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C39" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D39" s="13"/>
       <c r="E39" s="14"/>
@@ -1483,7 +1486,7 @@
         <v>1</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
@@ -1499,7 +1502,7 @@
         <v>1</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F43" s="4"/>
       <c r="G43" s="6"/>
@@ -1515,7 +1518,7 @@
         <v>1</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="6"/>
@@ -1531,7 +1534,7 @@
         <v>1</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
@@ -1547,7 +1550,7 @@
         <v>1</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
@@ -1563,7 +1566,7 @@
         <v>1</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" spans="3:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -1575,7 +1578,7 @@
         <v>1</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="49" spans="3:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -1587,7 +1590,7 @@
         <v>1</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="50" spans="3:12" ht="18" customHeight="1" x14ac:dyDescent="0.3">
@@ -1599,7 +1602,7 @@
         <v>6</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" spans="3:12" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1774,12 +1777,12 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>